<commit_message>
ajustando la carga por excel
</commit_message>
<xml_diff>
--- a/public/build/documentos/Importar-productos.xlsx
+++ b/public/build/documentos/Importar-productos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\contapos\public\build\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57B04D7A-B6D4-422A-B95E-F737FE0D90AE}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B33CA2B-CF01-424D-9CF7-52CEAAE8A379}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6300" yWindow="2190" windowWidth="24645" windowHeight="15645" xr2:uid="{04A6B785-A52E-42A5-AFDD-F9451D023F91}"/>
+    <workbookView xWindow="16380" yWindow="4260" windowWidth="24645" windowHeight="15645" xr2:uid="{04A6B785-A52E-42A5-AFDD-F9451D023F91}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>ID</t>
   </si>
@@ -65,7 +65,10 @@
     <t>PRECIO VENTA</t>
   </si>
   <si>
-    <t>stock</t>
+    <t>STOCK MINIMO</t>
+  </si>
+  <si>
+    <t>STOCK</t>
   </si>
 </sst>
 </file>
@@ -426,7 +429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{712CCE85-2FCD-41A1-A03B-72D1698EAE82}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -438,11 +441,12 @@
     <col min="8" max="8" width="8.42578125" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="8.5703125" customWidth="1"/>
-    <col min="11" max="11" width="17.28515625" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="11" max="11" width="15.140625" customWidth="1"/>
+    <col min="12" max="12" width="17" customWidth="1"/>
+    <col min="13" max="13" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -471,12 +475,15 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>